<commit_message>
Update BTC metrics: SL/TP and final decision - 2026-08-10 13:50:09.616088
</commit_message>
<xml_diff>
--- a/estrategia_reversion_a_media_resultados.xlsx
+++ b/estrategia_reversion_a_media_resultados.xlsx
@@ -1073,54 +1073,36 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>64496.53</v>
-      </c>
-      <c r="D10" t="n">
-        <v>62226.58</v>
-      </c>
-      <c r="E10" t="n">
-        <v>66694.64999999999</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>📦 ACUMULACIÓN/LATERAL</t>
-        </is>
-      </c>
+        <v>64496.15</v>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="n">
-        <v>64946.18</v>
-      </c>
-      <c r="I10" t="n">
-        <v>64339.53</v>
-      </c>
-      <c r="J10" t="n">
-        <v>63732.89</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>0.9708</v>
+      </c>
       <c r="N10" t="n">
         <v>-0.387</v>
       </c>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>⌀ BAJISTA</t>
-        </is>
-      </c>
+      <c r="O10" t="n">
+        <v>66921.41</v>
+      </c>
+      <c r="P10" t="n">
+        <v>59645.63</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>🔥 VENTA MAESTRA</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix: Forced Bitcoin visibility in Dashboard - 2026-08-10 13:50:17.537216
</commit_message>
<xml_diff>
--- a/estrategia_reversion_a_media_resultados.xlsx
+++ b/estrategia_reversion_a_media_resultados.xlsx
@@ -829,7 +829,7 @@
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>📈 BULL (Favorable)</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>📈 BULL (Favorable)</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>📉 BEAR (Presión)</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>📉 BEAR (Presión)</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update BTC: Added SL/TP and Beta metrics - 2026-08-10 13:50:27.781662
</commit_message>
<xml_diff>
--- a/estrategia_reversion_a_media_resultados.xlsx
+++ b/estrategia_reversion_a_media_resultados.xlsx
@@ -1242,9 +1242,15 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
+      <c r="N10" t="n">
+        <v>-0.387</v>
+      </c>
+      <c r="O10" t="n">
+        <v>66921.41</v>
+      </c>
+      <c r="P10" t="n">
+        <v>59645.63</v>
+      </c>
       <c r="Q10" t="inlineStr">
         <is>
           <t>🔥 VENTA MAESTRA</t>

</xml_diff>

<commit_message>
Update report: Bitcoin integration confirmed
</commit_message>
<xml_diff>
--- a/estrategia_reversion_a_media_resultados.xlsx
+++ b/estrategia_reversion_a_media_resultados.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel_Estrategico" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel_Maestro_Integral" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NZDUSD=X" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EURUSD=X" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JPY=X" sheetId="4" state="visible" r:id="rId4"/>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S10"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,72 +471,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Fibo 61.8%</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Fibo 38.2%</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Z-Score</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>R2_Optimizado</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Tendencia Predictiva</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
           <t>Decisión</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Stop Loss</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Take Profit</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Tendencia Actual del Mercado</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Sentimiento_Mercado</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>61.8%</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>50.0%</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>38.2%</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Señal_Sintética</t>
         </is>
       </c>
     </row>
@@ -552,50 +487,17 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.59</v>
+        <v>0.5885468721389771</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.5759904384613037</v>
       </c>
       <c r="E2" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1.16</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.8673</v>
-      </c>
-      <c r="J2" t="inlineStr">
+        <v>0.5908489227294922</v>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
-          <t>⌀ BAJISTA</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>📉 BEAR (Presión)</t>
-        </is>
-      </c>
-      <c r="L2" t="n">
-        <v>0.5911999999999999</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.5876</v>
-      </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>⚪ Neutral</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -611,50 +513,17 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.16</v>
+        <v>1.155001163482666</v>
       </c>
       <c r="D3" t="n">
-        <v>1.14</v>
+        <v>1.13544750213623</v>
       </c>
       <c r="E3" t="n">
-        <v>1.16</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="G3" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="H3" t="n">
-        <v>1.45</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.9005</v>
-      </c>
-      <c r="J3" t="inlineStr">
+        <v>1.157943487167358</v>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
-          <t>⌀ ALCISTA</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>📈 BULL (Favorable)</t>
-        </is>
-      </c>
-      <c r="L3" t="n">
-        <v>1.1377</v>
-      </c>
-      <c r="M3" t="n">
-        <v>1.2046</v>
-      </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>⚪ Neutral</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -670,50 +539,17 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>159.02</v>
+        <v>158.9629974365234</v>
       </c>
       <c r="D4" t="n">
-        <v>155.26</v>
+        <v>155.2559967041016</v>
       </c>
       <c r="E4" t="n">
-        <v>163.98</v>
-      </c>
-      <c r="F4" t="n">
-        <v>160.65</v>
-      </c>
-      <c r="G4" t="n">
-        <v>158.59</v>
-      </c>
-      <c r="H4" t="n">
-        <v>-0.96</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.8909</v>
-      </c>
-      <c r="J4" t="inlineStr">
+        <v>163.97900390625</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
-          <t>⌀ BAJISTA</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>📉 BEAR (Presión)</t>
-        </is>
-      </c>
-      <c r="L4" t="n">
-        <v>164.308</v>
-      </c>
-      <c r="M4" t="n">
-        <v>148.4441</v>
-      </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>⚪ Neutral</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -729,50 +565,17 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>29707.93</v>
+        <v>29750.5</v>
       </c>
       <c r="D5" t="n">
-        <v>27176.03</v>
+        <v>27176.029296875</v>
       </c>
       <c r="E5" t="n">
-        <v>30328.79</v>
-      </c>
-      <c r="F5" t="n">
-        <v>29124.43</v>
-      </c>
-      <c r="G5" t="n">
-        <v>28380.38</v>
-      </c>
-      <c r="H5" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.9683</v>
-      </c>
-      <c r="J5" t="inlineStr">
+        <v>29946.939453125</v>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
-          <t>⌀ ALCISTA</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>📈 BULL (Favorable)</t>
-        </is>
-      </c>
-      <c r="L5" t="n">
-        <v>27121.6779</v>
-      </c>
-      <c r="M5" t="n">
-        <v>34880.4341</v>
-      </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>⚪ Neutral</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -788,50 +591,17 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>7756.4</v>
+        <v>7761.81005859375</v>
       </c>
       <c r="D6" t="n">
-        <v>7313.92</v>
+        <v>7313.919921875</v>
       </c>
       <c r="E6" t="n">
-        <v>7793.68</v>
-      </c>
-      <c r="F6" t="n">
-        <v>7610.41</v>
-      </c>
-      <c r="G6" t="n">
-        <v>7497.19</v>
-      </c>
-      <c r="H6" t="n">
-        <v>1.63</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.9654</v>
-      </c>
-      <c r="J6" t="inlineStr">
+        <v>7793.68017578125</v>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
-          <t>⌀ ALCISTA</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>📈 BULL (Favorable)</t>
-        </is>
-      </c>
-      <c r="L6" t="n">
-        <v>7299.2922</v>
-      </c>
-      <c r="M6" t="n">
-        <v>8670.6157</v>
-      </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>⚪ Neutral</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -847,50 +617,17 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4394.7</v>
+        <v>4379.89990234375</v>
       </c>
       <c r="D7" t="n">
-        <v>3962.5</v>
+        <v>3964.199951171875</v>
       </c>
       <c r="E7" t="n">
         <v>4421.5</v>
       </c>
-      <c r="F7" t="n">
-        <v>4246.16</v>
-      </c>
-      <c r="G7" t="n">
-        <v>4137.84</v>
-      </c>
-      <c r="H7" t="n">
-        <v>2.57</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.9305</v>
-      </c>
-      <c r="J7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
-          <t>⌀ BAJISTA</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>⏳ BLOQUEO: Sobrecompra Extrema (No Comprar)</t>
-        </is>
-      </c>
-      <c r="L7" t="n">
-        <v>3962.5</v>
-      </c>
-      <c r="M7" t="n">
-        <v>4421.5</v>
-      </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>⚪ Neutral</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -906,50 +643,17 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>79.90000000000001</v>
+        <v>80.83000183105469</v>
       </c>
       <c r="D8" t="n">
-        <v>67.04000000000001</v>
+        <v>74.23999786376953</v>
       </c>
       <c r="E8" t="n">
         <v>93.5</v>
       </c>
-      <c r="F8" t="n">
-        <v>83.39</v>
-      </c>
-      <c r="G8" t="n">
-        <v>77.15000000000001</v>
-      </c>
-      <c r="H8" t="n">
-        <v>-0.46</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0.9396</v>
-      </c>
-      <c r="J8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
-          <t>⌀ BAJISTA</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>📉 BEAR (Presión)</t>
-        </is>
-      </c>
-      <c r="L8" t="n">
-        <v>93.687</v>
-      </c>
-      <c r="M8" t="n">
-        <v>52.326</v>
-      </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>⚪ Neutral</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -965,50 +669,17 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>64.31999999999999</v>
+        <v>63.91500091552734</v>
       </c>
       <c r="D9" t="n">
-        <v>55.01</v>
+        <v>55.01499938964844</v>
       </c>
       <c r="E9" t="n">
-        <v>65.05</v>
-      </c>
-      <c r="F9" t="n">
-        <v>61.22</v>
-      </c>
-      <c r="G9" t="n">
-        <v>58.85</v>
-      </c>
-      <c r="H9" t="n">
-        <v>2.33</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0.8752</v>
-      </c>
-      <c r="J9" t="inlineStr">
+        <v>65.05000305175781</v>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
-          <t>⌀ BAJISTA</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>⏳ BLOQUEO: Sobrecompra Extrema (No Comprar)</t>
-        </is>
-      </c>
-      <c r="L9" t="n">
-        <v>55.01</v>
-      </c>
-      <c r="M9" t="n">
-        <v>65.05</v>
-      </c>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>⚪ Neutral</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -1024,48 +695,17 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>64644.37</v>
+        <v>64644.37109375</v>
       </c>
       <c r="D10" t="n">
-        <v>62226.58</v>
+        <v>62226.578125</v>
       </c>
       <c r="E10" t="n">
-        <v>66694.64999999999</v>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr">
+        <v>66694.6484375</v>
+      </c>
+      <c r="F10" t="inlineStr">
         <is>
           <t>⚪ NEUTRAL</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>DISTRUBUCIÓN (TECHO)</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>Incertidumbre</t>
-        </is>
-      </c>
-      <c r="P10" t="n">
-        <v>73225.2328</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>70269.9883</v>
-      </c>
-      <c r="R10" t="n">
-        <v>67314.74370000001</v>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>📉 DISTRIBUCIÓN: Reducir Exposición</t>
         </is>
       </c>
     </row>
@@ -21600,7 +21240,7 @@
         <v>46244</v>
       </c>
       <c r="B260" t="n">
-        <v>0.58833909034729</v>
+        <v>0.5885468721389771</v>
       </c>
       <c r="C260" t="n">
         <v>0.5903884768486023</v>
@@ -21615,16 +21255,16 @@
         <v>0</v>
       </c>
       <c r="G260" t="n">
-        <v>0.5876501441001892</v>
+        <v>0.5876917004585266</v>
       </c>
       <c r="H260" t="n">
-        <v>0.5788361573219299</v>
+        <v>0.5788403129577637</v>
       </c>
       <c r="I260" t="n">
-        <v>0.582422502040863</v>
+        <v>0.5824245798587799</v>
       </c>
       <c r="J260" t="n">
-        <v>0.5826966717839241</v>
+        <v>0.5826977106928826</v>
       </c>
       <c r="K260" t="n">
         <v>0.004591460738863263</v>
@@ -30014,7 +29654,7 @@
         <v>1.157005667686462</v>
       </c>
       <c r="D260" t="n">
-        <v>1.154867768287659</v>
+        <v>1.154734373092651</v>
       </c>
       <c r="E260" t="n">
         <v>1.156738042831421</v>
@@ -38416,10 +38056,10 @@
         <v>46244</v>
       </c>
       <c r="B260" t="n">
-        <v>159.0229949951172</v>
+        <v>158.9629974365234</v>
       </c>
       <c r="C260" t="n">
-        <v>159.0379943847656</v>
+        <v>159.0639953613281</v>
       </c>
       <c r="D260" t="n">
         <v>157.5780029296875</v>
@@ -38431,19 +38071,19 @@
         <v>0</v>
       </c>
       <c r="G260" t="n">
-        <v>158.0506011962891</v>
+        <v>158.0386016845703</v>
       </c>
       <c r="H260" t="n">
-        <v>161.2294610595703</v>
+        <v>161.2282611083984</v>
       </c>
       <c r="I260" t="n">
-        <v>160.0150103759766</v>
+        <v>160.0144104003906</v>
       </c>
       <c r="J260" t="n">
-        <v>158.0652646636963</v>
+        <v>158.0649646759033</v>
       </c>
       <c r="K260" t="n">
-        <v>1.768214634486607</v>
+        <v>1.770071847098214</v>
       </c>
     </row>
   </sheetData>
@@ -46544,10 +46184,10 @@
         <v>46244</v>
       </c>
       <c r="B252" t="n">
-        <v>29707.9296875</v>
+        <v>29750.5</v>
       </c>
       <c r="C252" t="n">
-        <v>29730.3125</v>
+        <v>29750.5</v>
       </c>
       <c r="D252" t="n">
         <v>29610.015625</v>
@@ -46556,22 +46196,22 @@
         <v>29709.486328125</v>
       </c>
       <c r="F252" t="n">
-        <v>180861260</v>
+        <v>241887239</v>
       </c>
       <c r="G252" t="n">
-        <v>29604.901953125</v>
+        <v>29613.416015625</v>
       </c>
       <c r="H252" t="n">
-        <v>29358.9811328125</v>
+        <v>29359.8325390625</v>
       </c>
       <c r="I252" t="n">
-        <v>28038.4134375</v>
+        <v>28038.839140625</v>
       </c>
       <c r="J252" t="n">
-        <v>26647.39561523437</v>
+        <v>26647.60846679688</v>
       </c>
       <c r="K252" t="n">
-        <v>583.6432756696429</v>
+        <v>585.0852399553571</v>
       </c>
     </row>
   </sheetData>
@@ -54672,10 +54312,10 @@
         <v>46244</v>
       </c>
       <c r="B252" t="n">
-        <v>7756.39990234375</v>
+        <v>7761.81005859375</v>
       </c>
       <c r="C252" t="n">
-        <v>7761.43994140625</v>
+        <v>7762.66015625</v>
       </c>
       <c r="D252" t="n">
         <v>7748.419921875</v>
@@ -54684,22 +54324,22 @@
         <v>7751.740234375</v>
       </c>
       <c r="F252" t="n">
-        <v>289265170</v>
+        <v>406078665</v>
       </c>
       <c r="G252" t="n">
-        <v>7736.81396484375</v>
+        <v>7737.89599609375</v>
       </c>
       <c r="H252" t="n">
-        <v>7498.095615234375</v>
+        <v>7498.203818359375</v>
       </c>
       <c r="I252" t="n">
-        <v>7268.581025390625</v>
+        <v>7268.635126953125</v>
       </c>
       <c r="J252" t="n">
-        <v>7055.134953613281</v>
+        <v>7055.162004394531</v>
       </c>
       <c r="K252" t="n">
-        <v>88.469970703125</v>
+        <v>88.55712890625</v>
       </c>
     </row>
   </sheetData>
@@ -62800,7 +62440,7 @@
         <v>46244</v>
       </c>
       <c r="B252" t="n">
-        <v>4394.7001953125</v>
+        <v>4379.89990234375</v>
       </c>
       <c r="C252" t="n">
         <v>4421.5</v>
@@ -62812,19 +62452,19 @@
         <v>4400</v>
       </c>
       <c r="F252" t="n">
-        <v>61895</v>
+        <v>65664</v>
       </c>
       <c r="G252" t="n">
-        <v>4263.72001953125</v>
+        <v>4260.7599609375</v>
       </c>
       <c r="H252" t="n">
-        <v>4167.182021484375</v>
+        <v>4166.886015625</v>
       </c>
       <c r="I252" t="n">
-        <v>4402.02</v>
+        <v>4401.871997070312</v>
       </c>
       <c r="J252" t="n">
-        <v>4480.206490478516</v>
+        <v>4480.132489013672</v>
       </c>
       <c r="K252" t="n">
         <v>74.64283970424107</v>
@@ -70928,10 +70568,10 @@
         <v>46244</v>
       </c>
       <c r="B252" t="n">
-        <v>79.90000152587891</v>
+        <v>80.83000183105469</v>
       </c>
       <c r="C252" t="n">
-        <v>79.98000335693359</v>
+        <v>80.84999847412109</v>
       </c>
       <c r="D252" t="n">
         <v>77.79000091552734</v>
@@ -70940,22 +70580,22 @@
         <v>78.41999816894531</v>
       </c>
       <c r="F252" t="n">
-        <v>85965</v>
+        <v>97544</v>
       </c>
       <c r="G252" t="n">
-        <v>77.27200012207031</v>
+        <v>77.45800018310547</v>
       </c>
       <c r="H252" t="n">
-        <v>80.29020004272461</v>
+        <v>80.30880004882812</v>
       </c>
       <c r="I252" t="n">
-        <v>89.16639991760253</v>
+        <v>89.1756999206543</v>
       </c>
       <c r="J252" t="n">
-        <v>76.39099990844727</v>
+        <v>76.39564990997314</v>
       </c>
       <c r="K252" t="n">
-        <v>4.84857177734375</v>
+        <v>4.910714285714286</v>
       </c>
     </row>
   </sheetData>
@@ -79056,7 +78696,7 @@
         <v>46244</v>
       </c>
       <c r="B252" t="n">
-        <v>64.31500244140625</v>
+        <v>63.91500091552734</v>
       </c>
       <c r="C252" t="n">
         <v>64.62999725341797</v>
@@ -79068,19 +78708,19 @@
         <v>63.79999923706055</v>
       </c>
       <c r="F252" t="n">
-        <v>17653</v>
+        <v>18836</v>
       </c>
       <c r="G252" t="n">
-        <v>62.24820022583008</v>
+        <v>62.1681999206543</v>
       </c>
       <c r="H252" t="n">
-        <v>62.56325973510742</v>
+        <v>62.55525970458984</v>
       </c>
       <c r="I252" t="n">
-        <v>69.2087596130371</v>
+        <v>69.20475959777832</v>
       </c>
       <c r="J252" t="n">
-        <v>70.22765995025635</v>
+        <v>70.22565994262695</v>
       </c>
       <c r="K252" t="n">
         <v>1.483785629272461</v>

</xml_diff>

<commit_message>
Update BTC metrics: SL/TP and final decision - 2026-08-10 14:14:08.605089
</commit_message>
<xml_diff>
--- a/estrategia_reversion_a_media_resultados.xlsx
+++ b/estrategia_reversion_a_media_resultados.xlsx
@@ -1073,54 +1073,36 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>64637.52</v>
-      </c>
-      <c r="D10" t="n">
-        <v>62226.58</v>
-      </c>
-      <c r="E10" t="n">
-        <v>66694.64999999999</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>📦 ACUMULACIÓN/LATERAL</t>
-        </is>
-      </c>
+        <v>64637.54</v>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="n">
-        <v>64946.18</v>
-      </c>
-      <c r="I10" t="n">
-        <v>64339.53</v>
-      </c>
-      <c r="J10" t="n">
-        <v>63732.89</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>0.9708</v>
+      </c>
       <c r="N10" t="n">
         <v>-0.3881</v>
       </c>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>⌀ BAJISTA</t>
-        </is>
-      </c>
+      <c r="O10" t="n">
+        <v>67072.53999999999</v>
+      </c>
+      <c r="P10" t="n">
+        <v>59767.54</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>🔥 VENTA MAESTRA</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix: Forced Bitcoin visibility in Dashboard - 2026-08-10 14:14:16.345727
</commit_message>
<xml_diff>
--- a/estrategia_reversion_a_media_resultados.xlsx
+++ b/estrategia_reversion_a_media_resultados.xlsx
@@ -829,7 +829,7 @@
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>📈 BULL (Favorable)</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>📈 BULL (Favorable)</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>📉 BEAR (Presión)</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -1045,7 +1045,7 @@
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>📈 BULL (Favorable)</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>📉 BEAR (Presión)</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update BTC: Added SL/TP and Beta metrics - 2026-08-10 14:14:27.214080
</commit_message>
<xml_diff>
--- a/estrategia_reversion_a_media_resultados.xlsx
+++ b/estrategia_reversion_a_media_resultados.xlsx
@@ -1242,9 +1242,15 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
+      <c r="N10" t="n">
+        <v>-0.3881</v>
+      </c>
+      <c r="O10" t="n">
+        <v>67072.53999999999</v>
+      </c>
+      <c r="P10" t="n">
+        <v>59767.54</v>
+      </c>
       <c r="Q10" t="inlineStr">
         <is>
           <t>🔥 VENTA MAESTRA</t>

</xml_diff>

<commit_message>
Update BTC metrics: SL/TP and final decision - 2026-08-10 15:13:14.962577
</commit_message>
<xml_diff>
--- a/estrategia_reversion_a_media_resultados.xlsx
+++ b/estrategia_reversion_a_media_resultados.xlsx
@@ -1073,54 +1073,36 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>64505.11</v>
-      </c>
-      <c r="D10" t="n">
-        <v>62226.58</v>
-      </c>
-      <c r="E10" t="n">
-        <v>66694.64999999999</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>📦 ACUMULACIÓN/LATERAL</t>
-        </is>
-      </c>
+        <v>64494.49</v>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="n">
-        <v>64946.18</v>
-      </c>
-      <c r="I10" t="n">
-        <v>64339.53</v>
-      </c>
-      <c r="J10" t="n">
-        <v>63732.89</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>0.9708</v>
+      </c>
       <c r="N10" t="n">
         <v>-0.3871</v>
       </c>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>⌀ BAJISTA</t>
-        </is>
-      </c>
+      <c r="O10" t="n">
+        <v>66929.49000000001</v>
+      </c>
+      <c r="P10" t="n">
+        <v>59624.49</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>🔥 VENTA MAESTRA</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix: Forced Bitcoin visibility in Dashboard - 2026-08-10 15:13:22.219235
</commit_message>
<xml_diff>
--- a/estrategia_reversion_a_media_resultados.xlsx
+++ b/estrategia_reversion_a_media_resultados.xlsx
@@ -829,7 +829,7 @@
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>📈 BULL (Favorable)</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>📈 BULL (Favorable)</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>📉 BEAR (Presión)</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -1045,7 +1045,7 @@
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>📈 BULL (Favorable)</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>📉 BEAR (Presión)</t>
+          <t>⚪ NEUTRAL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update BTC: Added SL/TP and Beta metrics - 2026-08-10 15:13:34.320484
</commit_message>
<xml_diff>
--- a/estrategia_reversion_a_media_resultados.xlsx
+++ b/estrategia_reversion_a_media_resultados.xlsx
@@ -1242,9 +1242,15 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
+      <c r="N10" t="n">
+        <v>-0.3871</v>
+      </c>
+      <c r="O10" t="n">
+        <v>66929.49000000001</v>
+      </c>
+      <c r="P10" t="n">
+        <v>59624.49</v>
+      </c>
       <c r="Q10" t="inlineStr">
         <is>
           <t>🔥 VENTA MAESTRA</t>

</xml_diff>